<commit_message>
Updating with previous work from earlier in the year.
</commit_message>
<xml_diff>
--- a/data/nodes.xlsx
+++ b/data/nodes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\CSAM-deployment-optimization\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F62C9530-4BD8-459F-8DBC-95300EBA720B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C704321A-C5FA-4BF9-B263-D8313324945B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="360" windowWidth="29040" windowHeight="15720" xr2:uid="{70223939-7149-498B-8718-169659C9181E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{70223939-7149-498B-8718-169659C9181E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>node</t>
   </si>
@@ -57,25 +57,70 @@
   </si>
   <si>
     <t>exercise</t>
+  </si>
+  <si>
+    <t>Misawa_AB</t>
+  </si>
+  <si>
+    <t>Yokota_AB</t>
+  </si>
+  <si>
+    <t>Zama_Camp</t>
+  </si>
+  <si>
+    <t>Atsugi_NAS</t>
+  </si>
+  <si>
+    <t>Yokosuka_NFA</t>
+  </si>
+  <si>
+    <t>Iwakuni_MCAS</t>
+  </si>
+  <si>
+    <t>Sasebo_NFA</t>
+  </si>
+  <si>
+    <t>Fuji_Camp</t>
+  </si>
+  <si>
+    <t>Suwon_AB</t>
+  </si>
+  <si>
+    <t>Osan_AB</t>
+  </si>
+  <si>
+    <t>Kunsan_AB</t>
+  </si>
+  <si>
+    <t>Humphreys_Camp</t>
+  </si>
+  <si>
+    <t>Walker_Camp</t>
+  </si>
+  <si>
+    <t>Mujuk_Camp</t>
+  </si>
+  <si>
+    <t>Pohang_AB</t>
+  </si>
+  <si>
+    <t>Jeju_Port</t>
+  </si>
+  <si>
+    <t>Taegu_AB</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="16"/>
-      <color rgb="FF000000"/>
-      <name val="Rubik"/>
     </font>
   </fonts>
   <fills count="2">
@@ -98,9 +143,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -435,14 +479,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37F740F8-50EF-4B32-9A42-8A925D4FCB56}">
-  <dimension ref="A1:G2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:G18"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="5" max="5" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.42578125" customWidth="1"/>
+    <col min="6" max="6" width="12.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -465,8 +510,90 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="20.25">
-      <c r="A2" s="1"/>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>23</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>